<commit_message>
feat: add VerifierDisponibiliteAgenda workflow and associated data files
</commit_message>
<xml_diff>
--- a/Data/Agenda_Medecin.xlsx
+++ b/Data/Agenda_Medecin.xlsx
@@ -82,6 +82,9 @@
     <x:t>11:00</x:t>
   </x:si>
   <x:si>
+    <x:t>Libre</x:t>
+  </x:si>
+  <x:si>
     <x:t>AG-006</x:t>
   </x:si>
   <x:si>
@@ -106,16 +109,19 @@
     <x:t>AG-009</x:t>
   </x:si>
   <x:si>
-    <x:t>Libre</x:t>
+    <x:t>Laith Mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Consultation générale</x:t>
   </x:si>
   <x:si>
     <x:t>AG-010</x:t>
   </x:si>
   <x:si>
-    <x:t>Laith Mahdi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Consultation générale</x:t>
+    <x:t>Dalel Loussaief</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Renouvellement ordonnance</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -269,22 +275,22 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="20" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -771,10 +777,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="E6" s="11" t="s">
-        <x:v>10</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F6" s="11" t="s">
-        <x:v>10</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G6" s="11" t="s">
         <x:v>10</x:v>
@@ -782,16 +788,16 @@
     </x:row>
     <x:row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A7" s="14" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B7" s="15">
         <x:v>46141</x:v>
       </x:c>
       <x:c r="C7" s="14" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="16" t="s">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E7" s="14" t="s">
         <x:v>10</x:v>
@@ -805,16 +811,16 @@
     </x:row>
     <x:row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A8" s="11" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B8" s="12">
         <x:v>46141</x:v>
       </x:c>
       <x:c r="C8" s="11" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D8" s="16" t="s">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E8" s="11" t="s">
         <x:v>10</x:v>
@@ -828,16 +834,16 @@
     </x:row>
     <x:row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A9" s="14" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B9" s="15">
         <x:v>46141</x:v>
       </x:c>
       <x:c r="C9" s="14" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D9" s="17" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E9" s="14" t="s">
         <x:v>10</x:v>
@@ -851,7 +857,7 @@
     </x:row>
     <x:row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A10" s="11" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B10" s="12">
         <x:v>46141</x:v>
@@ -863,10 +869,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="E10" s="11" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="s">
-        <x:v>31</x:v>
       </x:c>
       <x:c r="G10" s="11" t="s">
         <x:v>10</x:v>
@@ -874,7 +880,7 @@
     </x:row>
     <x:row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A11" s="14" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B11" s="15">
         <x:v>46142</x:v>
@@ -883,7 +889,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D11" s="16" t="s">
-        <x:v>28</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E11" s="14" t="s">
         <x:v>10</x:v>

</xml_diff>

<commit_message>
feat: implement API routes for patient login and appointment management with Swagger documentation
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Data/Agenda_Medecin.xlsx
+++ b/Data/Agenda_Medecin.xlsx
@@ -49,19 +49,25 @@
     <x:t>09:00</x:t>
   </x:si>
   <x:si>
+    <x:t>Libre</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>AG-002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09:30</x:t>
+  </x:si>
+  <x:si>
     <x:t>Réservé</x:t>
   </x:si>
   <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>AG-002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09:30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Occupé</x:t>
+    <x:t>Laith Mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Consultation générale</x:t>
   </x:si>
   <x:si>
     <x:t>AG-003</x:t>
@@ -88,9 +94,6 @@
     <x:t>11:30</x:t>
   </x:si>
   <x:si>
-    <x:t>Libre</x:t>
-  </x:si>
-  <x:si>
     <x:t>AG-007</x:t>
   </x:si>
   <x:si>
@@ -103,22 +106,13 @@
     <x:t>14:30</x:t>
   </x:si>
   <x:si>
-    <x:t>Bloqué</x:t>
-  </x:si>
-  <x:si>
     <x:t>AG-009</x:t>
   </x:si>
   <x:si>
-    <x:t>Laith Mahdi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Consultation générale</x:t>
-  </x:si>
-  <x:si>
     <x:t>AG-010</x:t>
   </x:si>
   <x:si>
-    <x:t>Mahdi Leith</x:t>
+    <x:t>Mahdy Leith</x:t>
   </x:si>
   <x:si>
     <x:t>Résultat analyses</x:t>
@@ -131,7 +125,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="7" x14ac:knownFonts="1">
+  <x:fonts count="5" x14ac:knownFonts="1">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -150,22 +144,11 @@
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF1565C0"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF006100"/>
       <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF2E7D32"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FFC62828"/>
-      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
     </x:font>
     <x:font>
       <x:vertAlign val="baseline"/>
@@ -175,7 +158,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -194,22 +177,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFBBDEFB"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF5F5F5"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFC8E6C9"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFCDD2"/>
+        <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -237,8 +210,9 @@
       <x:diagonal/>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="11">
+  <x:cellStyleXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -248,29 +222,23 @@
     <x:xf numFmtId="14" fontId="2" fillId="3" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="2" fillId="5" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="14" fontId="2" fillId="4" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="20" fontId="2" fillId="3" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="20" fontId="2" fillId="5" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="20" fontId="2" fillId="4" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -281,25 +249,19 @@
     <x:xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="14" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="20" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="20" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="20" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -314,23 +276,15 @@
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="14" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -338,12 +292,13 @@
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="20" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="20" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="1">
+  <x:cellStyles count="2">
+    <x:cellStyle name="Good" xfId="1" builtinId="26"/>
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
   </x:cellStyles>
   <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -659,255 +614,255 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A1" s="11" t="s">
+      <x:c r="A1" s="9" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="11" t="s">
+      <x:c r="B1" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="11" t="s">
+      <x:c r="C1" s="9" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="11" t="s">
+      <x:c r="D1" s="9" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E1" s="11" t="s">
+      <x:c r="E1" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F1" s="11" t="s">
+      <x:c r="F1" s="9" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G1" s="11" t="s">
+      <x:c r="G1" s="9" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A2" s="12" t="s">
+      <x:c r="A2" s="10" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B2" s="13">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C2" s="12" t="s">
+      <x:c r="B2" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D2" s="14" t="s">
+      <x:c r="D2" s="12" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E2" s="10" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F2" s="10" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G2" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A3" s="13" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B3" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C3" s="13" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E3" s="13" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G3" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A4" s="10" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B4" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E2" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F2" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G2" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A3" s="15" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B3" s="16">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C3" s="15" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E3" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F3" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G3" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A4" s="12" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B4" s="13">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D4" s="17" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="s">
+      <x:c r="E4" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A5" s="15" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B5" s="16">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C5" s="15" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="D5" s="14" t="s">
+      <x:c r="A5" s="13" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B5" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E5" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F5" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G5" s="15" t="s">
+      <x:c r="E5" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G5" s="13" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A6" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B6" s="13">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C6" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D6" s="17" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E6" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F6" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G6" s="12" t="s">
+      <x:c r="A6" s="10" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B6" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A7" s="15" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B7" s="16">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C7" s="15" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D7" s="17" t="s">
+      <x:c r="A7" s="13" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E7" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F7" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G7" s="15" t="s">
+      <x:c r="B7" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E7" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G7" s="13" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A8" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B8" s="13">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C8" s="12" t="s">
+      <x:c r="A8" s="10" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="D8" s="17" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F8" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G8" s="12" t="s">
+      <x:c r="B8" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A9" s="15" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B9" s="16">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C9" s="15" t="s">
+      <x:c r="A9" s="13" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D9" s="18" t="s">
+      <x:c r="B9" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E9" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F9" s="15" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G9" s="15" t="s">
+      <x:c r="D9" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F9" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A10" s="12" t="s">
+      <x:c r="A10" s="10" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B10" s="13">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C10" s="19">
+      <x:c r="B10" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C10" s="15">
         <x:v>0.625</x:v>
       </x:c>
-      <x:c r="D10" s="17" t="s">
+      <x:c r="D10" s="12" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E10" s="12" t="s">
+      <x:c r="E10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A11" s="13" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="F10" s="12" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G10" s="12" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <x:c r="A11" s="15" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B11" s="16">
-        <x:v>46141</x:v>
-      </x:c>
-      <x:c r="C11" s="20">
+      <x:c r="B11" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C11" s="16">
         <x:v>0.645833333333333</x:v>
       </x:c>
-      <x:c r="D11" s="17" t="s">
+      <x:c r="D11" s="12" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E11" s="15" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F11" s="15" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="G11" s="15" t="s">
+      <x:c r="E11" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: add RPA project data files and initial technical documentation
</commit_message>
<xml_diff>
--- a/Data/Agenda_Medecin.xlsx
+++ b/Data/Agenda_Medecin.xlsx
@@ -13,6 +13,7 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Agenda" sheetId="1" r:id="rId1"/>
+    <x:sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="0"/>
@@ -61,6 +62,12 @@
     <x:t>09:30</x:t>
   </x:si>
   <x:si>
+    <x:t>AG-003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10:00</x:t>
+  </x:si>
+  <x:si>
     <x:t>Réservé</x:t>
   </x:si>
   <x:si>
@@ -70,12 +77,6 @@
     <x:t>Consultation générale</x:t>
   </x:si>
   <x:si>
-    <x:t>AG-003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:00</x:t>
-  </x:si>
-  <x:si>
     <x:t>AG-004</x:t>
   </x:si>
   <x:si>
@@ -116,6 +117,9 @@
   </x:si>
   <x:si>
     <x:t>Résultat analyses</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mahdy Leyth</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -210,9 +214,8 @@
       <x:diagonal/>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="10">
+  <x:cellStyleXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -249,6 +252,9 @@
     <x:xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
@@ -261,9 +267,6 @@
     <x:xf numFmtId="20" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -297,8 +300,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="2">
-    <x:cellStyle name="Good" xfId="1" builtinId="26"/>
+  <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
   </x:cellStyles>
   <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -647,13 +649,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="12" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="10" t="s">
-        <x:v>30</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="10" t="s">
-        <x:v>31</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G2" s="10" t="s">
         <x:v>10</x:v>
@@ -670,13 +672,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D3" s="12" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E3" s="13" t="s">
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="13" t="s">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
         <x:v>10</x:v>
@@ -684,22 +686,22 @@
     </x:row>
     <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A4" s="10" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B4" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B4" s="11">
-        <x:v>46142</x:v>
-      </x:c>
-      <x:c r="C4" s="10" t="s">
+      <x:c r="F4" s="10" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E4" s="10" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F4" s="10" t="s">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="G4" s="10" t="s">
         <x:v>10</x:v>
@@ -716,13 +718,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="12" t="s">
-        <x:v>9</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="13" t="s">
-        <x:v>10</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F5" s="13" t="s">
-        <x:v>10</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G5" s="13" t="s">
         <x:v>10</x:v>
@@ -873,4 +875,278 @@
   <x:headerFooter/>
   <x:tableParts count="0"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:G11"/>
+  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.285156" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A1" s="9" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="9" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="9" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B2" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E2" s="10" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F2" s="10" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G2" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A3" s="13" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B3" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C3" s="13" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E3" s="13" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G3" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A4" s="10" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B4" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A5" s="13" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B5" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E5" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G5" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A6" s="10" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B6" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A7" s="13" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B7" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E7" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G7" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A8" s="10" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B8" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A9" s="13" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B9" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E9" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F9" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A10" s="10" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B10" s="11">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C10" s="15">
+        <x:v>0.625</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <x:c r="A11" s="13" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B11" s="14">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C11" s="16">
+        <x:v>0.645833333333333</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>